<commit_message>
transform adapted, extended to STAP, deregularisation update, TARSP form update
</commit_message>
<xml_diff>
--- a/src/sastadev/data/form_templates/TARSP Form Current.xlsx
+++ b/src/sastadev/data/form_templates/TARSP Form Current.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22527"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\jodijk\Dropbox\jodijk\Utrecht\Projects\CLARIAH CORE\WP3\VKL\TARSP\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\jodijk\myprograms\python\sastacode\mysastadev\src\sastadev\data\form_templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F977736-91AA-4CB3-8297-ECE5E2C017EA}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DE1A580-C17E-4E37-921A-E01F11673F1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{264B2C4D-E364-489B-B80A-827BE72E938B}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{264B2C4D-E364-489B-B80A-827BE72E938B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="373" uniqueCount="367">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="379" uniqueCount="373">
   <si>
     <t>Naam</t>
   </si>
@@ -1134,6 +1134,24 @@
   </si>
   <si>
     <t>T066c</t>
+  </si>
+  <si>
+    <t>T003</t>
+  </si>
+  <si>
+    <t>T003c</t>
+  </si>
+  <si>
+    <t>T098</t>
+  </si>
+  <si>
+    <t>T098c</t>
+  </si>
+  <si>
+    <t>T060</t>
+  </si>
+  <si>
+    <t>T060c</t>
   </si>
 </sst>
 </file>
@@ -1204,9 +1222,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1244,7 +1262,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1350,7 +1368,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1492,7 +1510,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -2448,6 +2466,12 @@
       <c r="B46" t="s">
         <v>113</v>
       </c>
+      <c r="C46" t="s">
+        <v>371</v>
+      </c>
+      <c r="D46" t="s">
+        <v>372</v>
+      </c>
     </row>
     <row r="47" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A47">
@@ -2479,6 +2503,12 @@
       <c r="B48" t="s">
         <v>114</v>
       </c>
+      <c r="C48" t="s">
+        <v>367</v>
+      </c>
+      <c r="D48" t="s">
+        <v>368</v>
+      </c>
       <c r="N48" t="s">
         <v>120</v>
       </c>
@@ -2498,6 +2528,12 @@
       </c>
       <c r="B49" t="s">
         <v>115</v>
+      </c>
+      <c r="C49" t="s">
+        <v>369</v>
+      </c>
+      <c r="D49" t="s">
+        <v>370</v>
       </c>
       <c r="N49" t="s">
         <v>121</v>

</xml_diff>

<commit_message>
improvements of TARSP form
</commit_message>
<xml_diff>
--- a/src/sastadev/data/form_templates/TARSP Form Current.xlsx
+++ b/src/sastadev/data/form_templates/TARSP Form Current.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\jodijk\myprograms\python\sastacode\mysastadev\src\sastadev\data\form_templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DE1A580-C17E-4E37-921A-E01F11673F1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FF6CDF7-B61E-44D4-A97E-09C18ED0EDD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{264B2C4D-E364-489B-B80A-827BE72E938B}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{264B2C4D-E364-489B-B80A-827BE72E938B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="379" uniqueCount="373">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="384" uniqueCount="378">
   <si>
     <t>Naam</t>
   </si>
@@ -1152,6 +1152,21 @@
   </si>
   <si>
     <t>T060c</t>
+  </si>
+  <si>
+    <t>T156</t>
+  </si>
+  <si>
+    <t>T156c</t>
+  </si>
+  <si>
+    <t>T049</t>
+  </si>
+  <si>
+    <t>T049c</t>
+  </si>
+  <si>
+    <t>T151</t>
   </si>
 </sst>
 </file>
@@ -1635,6 +1650,9 @@
       <c r="W8" s="1" t="s">
         <v>25</v>
       </c>
+      <c r="X8" t="s">
+        <v>377</v>
+      </c>
     </row>
     <row r="9" spans="1:26" x14ac:dyDescent="0.3">
       <c r="C9" t="s">
@@ -1938,6 +1956,12 @@
       <c r="E25" t="s">
         <v>61</v>
       </c>
+      <c r="F25" t="s">
+        <v>375</v>
+      </c>
+      <c r="G25" t="s">
+        <v>376</v>
+      </c>
       <c r="N25" t="s">
         <v>66</v>
       </c>
@@ -2309,6 +2333,12 @@
       </c>
       <c r="N40" t="s">
         <v>47</v>
+      </c>
+      <c r="O40" t="s">
+        <v>373</v>
+      </c>
+      <c r="P40" t="s">
+        <v>374</v>
       </c>
     </row>
     <row r="41" spans="1:25" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
form toelichting PF & TARSP-P
</commit_message>
<xml_diff>
--- a/src/sastadev/data/form_templates/TARSP Form Current.xlsx
+++ b/src/sastadev/data/form_templates/TARSP Form Current.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\jodijk\myprograms\python\sastacode\mysastadev\src\sastadev\data\form_templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FF6CDF7-B61E-44D4-A97E-09C18ED0EDD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2BEB070-FE02-477A-BC4A-D95F16115C09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{264B2C4D-E364-489B-B80A-827BE72E938B}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{264B2C4D-E364-489B-B80A-827BE72E938B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -2432,13 +2432,13 @@
       <c r="D44" t="s">
         <v>283</v>
       </c>
-      <c r="E44" t="s">
+      <c r="H44" t="s">
         <v>103</v>
       </c>
-      <c r="F44" t="s">
+      <c r="I44" t="s">
         <v>284</v>
       </c>
-      <c r="G44" t="s">
+      <c r="J44" t="s">
         <v>285</v>
       </c>
       <c r="N44" t="s">
@@ -2461,13 +2461,13 @@
       <c r="D45" t="s">
         <v>289</v>
       </c>
-      <c r="E45" t="s">
+      <c r="H45" t="s">
         <v>104</v>
       </c>
-      <c r="F45" t="s">
+      <c r="I45" t="s">
         <v>286</v>
       </c>
-      <c r="G45" t="s">
+      <c r="J45" t="s">
         <v>287</v>
       </c>
       <c r="K45" t="s">
@@ -2672,13 +2672,13 @@
       </c>
     </row>
     <row r="53" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="E53" t="s">
+      <c r="H53" t="s">
         <v>117</v>
       </c>
-      <c r="F53" t="s">
+      <c r="I53" t="s">
         <v>358</v>
       </c>
-      <c r="G53" t="s">
+      <c r="J53" t="s">
         <v>359</v>
       </c>
       <c r="N53" t="s">
@@ -2701,13 +2701,13 @@
       </c>
     </row>
     <row r="54" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="E54" t="s">
+      <c r="H54" t="s">
         <v>118</v>
       </c>
-      <c r="F54" t="s">
+      <c r="I54" t="s">
         <v>356</v>
       </c>
-      <c r="G54" t="s">
+      <c r="J54" t="s">
         <v>357</v>
       </c>
       <c r="K54" t="s">

</xml_diff>